<commit_message>
Rename simulated CEO to Jerry Gold across reports, data, PDFs and workbooks
</commit_message>
<xml_diff>
--- a/01-security-policy-pack/01-policy-signoff-tracker.xlsx
+++ b/01-security-policy-pack/01-policy-signoff-tracker.xlsx
@@ -51,7 +51,7 @@
     <t xml:space="preserve">Approved by</t>
   </si>
   <si>
-    <t xml:space="preserve">Jerry Olugboye, Chief Executive Officer</t>
+    <t xml:space="preserve">Jerry Gold, Chief Executive Officer</t>
   </si>
   <si>
     <t xml:space="preserve">Classification</t>
@@ -225,7 +225,7 @@
     <t xml:space="preserve">Hardware Key</t>
   </si>
   <si>
-    <t xml:space="preserve">Jerry Olugboye</t>
+    <t xml:space="preserve">Jerry Gold</t>
   </si>
   <si>
     <t xml:space="preserve">CGI-027</t>

</xml_diff>